<commit_message>
- Added method Insert-To-Cells that replace all cells containing a specified string value with the desired one - Removed AutoFitColumns to prevent it from affecting templates
</commit_message>
<xml_diff>
--- a/XporterConsole/Templates/templ.xlsx
+++ b/XporterConsole/Templates/templ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dgrevenos\source\repos\Xporter\XporterConsole\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mitsos\source\repos\Xporter\XporterConsole\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB48C04-9218-41C8-AEA6-17FD8535E8E3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD11DB73-ABAF-44CD-A34B-73E5874ACD0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5685" yWindow="4200" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Templ" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="8">
   <si>
     <t>MMPublication</t>
   </si>
@@ -38,6 +38,18 @@
   </si>
   <si>
     <t>Template Ex.</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>asdf</t>
+  </si>
+  <si>
+    <t>asdfasdfasdfasdfa</t>
+  </si>
+  <si>
+    <t>asdfasdfasdfasdf</t>
   </si>
 </sst>
 </file>
@@ -223,7 +235,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -514,59 +526,349 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Q22"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="13" customWidth="1"/>
-    <col min="2" max="2" width="30.5546875" style="13" customWidth="1"/>
+    <col min="2" max="2" width="30.5703125" style="13" customWidth="1"/>
     <col min="3" max="3" width="30" style="13" customWidth="1"/>
-    <col min="4" max="4" width="27.77734375" style="13" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="13"/>
+    <col min="4" max="4" width="27.7109375" style="13" customWidth="1"/>
+    <col min="5" max="16384" width="8.85546875" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="36.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:15" ht="36.75" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4"/>
     </row>
-    <row r="2" spans="1:2" ht="24.6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:15" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A2" s="5"/>
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="6"/>
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:2" ht="18.600000000000001" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="8"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="11"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="6"/>
       <c r="B5" s="2"/>
-    </row>
-    <row r="6" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="11"/>
+    </row>
+    <row r="6" spans="1:15" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="10"/>
-    </row>
-    <row r="9" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="17" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="18" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="19" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="20" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="21" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+      <c r="N6" s="11"/>
+      <c r="O6" s="11"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11"/>
+      <c r="O7" s="11"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="11"/>
+    </row>
+    <row r="9" spans="1:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11"/>
+    </row>
+    <row r="10" spans="1:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+    </row>
+    <row r="11" spans="1:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+    </row>
+    <row r="12" spans="1:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+    </row>
+    <row r="13" spans="1:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="11"/>
+    </row>
+    <row r="14" spans="1:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+    </row>
+    <row r="15" spans="1:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="11"/>
+    </row>
+    <row r="16" spans="1:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="11"/>
+    </row>
+    <row r="17" spans="2:17" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="11"/>
+    </row>
+    <row r="18" spans="2:17" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="N18" s="11"/>
+      <c r="O18" s="11"/>
+    </row>
+    <row r="19" spans="2:17" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="11"/>
+      <c r="N19" s="11"/>
+      <c r="O19" s="11"/>
+    </row>
+    <row r="20" spans="2:17" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="11"/>
+      <c r="N20" s="11"/>
+      <c r="O20" s="11"/>
+    </row>
+    <row r="21" spans="2:17" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="11"/>
+      <c r="N21" s="11"/>
+      <c r="O21" s="11"/>
+    </row>
+    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="11"/>
+      <c r="N22" s="11"/>
+      <c r="O22" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="P22" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q22" s="13" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -576,88 +878,104 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91727B64-FB78-401B-8250-2F293487328F}">
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O22"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="11" customWidth="1"/>
-    <col min="2" max="2" width="30.5546875" style="11" customWidth="1"/>
+    <col min="2" max="2" width="30.5703125" style="11" customWidth="1"/>
     <col min="3" max="3" width="30" style="11" customWidth="1"/>
-    <col min="4" max="4" width="27.77734375" style="11" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="11"/>
+    <col min="4" max="4" width="27.7109375" style="11" customWidth="1"/>
+    <col min="5" max="16384" width="8.85546875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="36.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:9" ht="36.75" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="4"/>
     </row>
-    <row r="2" spans="1:4" ht="24.6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A2" s="5"/>
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="6"/>
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:4" ht="18.600000000000001" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="8"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="6"/>
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="10"/>
       <c r="D6" s="12"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C8" s="13"/>
     </row>
-    <row r="9" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="13"/>
-    </row>
-    <row r="10" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F9" s="11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="13"/>
     </row>
-    <row r="11" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="13"/>
     </row>
-    <row r="12" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="13"/>
     </row>
-    <row r="13" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="13"/>
-    </row>
-    <row r="14" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I13" s="11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="13"/>
     </row>
-    <row r="15" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="13"/>
     </row>
-    <row r="16" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="13"/>
     </row>
-    <row r="17" spans="3:3" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="13"/>
     </row>
-    <row r="18" spans="3:3" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="13"/>
-    </row>
-    <row r="19" spans="3:3" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L18" s="11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="3:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="13"/>
     </row>
-    <row r="20" spans="3:3" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="13"/>
     </row>
-    <row r="21" spans="3:3" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:15" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="13"/>
+    </row>
+    <row r="22" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="O22" s="11" t="s">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>